<commit_message>
CopyCellValue() fully implemented, manage also currencies
</commit_message>
<xml_diff>
--- a/3-Dev/DevApp/Files/currencies.xlsx
+++ b/3-Dev/DevApp/Files/currencies.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a990f455bb745add/ProjetsDev/10-Pierlam/OpenExcelSdk/Dev/OpenExcelSdk/3-Dev/DevApp/Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="69" documentId="11_AD4DB114E441178AC67DF4536695FF58683EDF1B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{865D4EA1-D65F-41EB-9481-F3CC6CD62351}"/>
+  <xr:revisionPtr revIDLastSave="70" documentId="11_AD4DB114E441178AC67DF4536695FF58683EDF1B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B3A58099-1A77-4C3A-9676-397EAA569E0C}"/>
   <bookViews>
-    <workbookView xWindow="1755" yWindow="2160" windowWidth="23925" windowHeight="13350" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6555" yWindow="2010" windowWidth="21075" windowHeight="13350" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sheet1" sheetId="1" r:id="rId1"/>
@@ -84,9 +84,9 @@
     <numFmt numFmtId="173" formatCode="_ [$¥-804]* #,##0.00_ ;_ [$¥-804]* \-#,##0.00_ ;_ [$¥-804]* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="174" formatCode="[$¥-804]#,##0.00"/>
     <numFmt numFmtId="175" formatCode="[$£-809]#,##0.00"/>
-    <numFmt numFmtId="177" formatCode="#,##0.00\ [$CHF-417]"/>
-    <numFmt numFmtId="178" formatCode="[$¥-411]#,##0.00"/>
-    <numFmt numFmtId="179" formatCode="[$₩-412]#,##0.00"/>
+    <numFmt numFmtId="176" formatCode="#,##0.00\ [$CHF-417]"/>
+    <numFmt numFmtId="177" formatCode="[$¥-411]#,##0.00"/>
+    <numFmt numFmtId="178" formatCode="[$₩-412]#,##0.00"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -132,9 +132,9 @@
     <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="175" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -423,7 +423,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" customWidth="1"/>
+    <col min="2" max="2" width="24.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
focus on currency get/set
</commit_message>
<xml_diff>
--- a/3-Dev/DevApp/Files/currencies.xlsx
+++ b/3-Dev/DevApp/Files/currencies.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a990f455bb745add/ProjetsDev/10-Pierlam/OpenExcelSdk/Dev/OpenExcelSdk/3-Dev/DevApp/Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="70" documentId="11_AD4DB114E441178AC67DF4536695FF58683EDF1B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B3A58099-1A77-4C3A-9676-397EAA569E0C}"/>
+  <xr:revisionPtr revIDLastSave="108" documentId="11_AD4DB114E441178AC67DF4536695FF58683EDF1B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8BB245D-BB90-4605-9BCB-899E3F331D65}"/>
   <bookViews>
-    <workbookView xWindow="6555" yWindow="2010" windowWidth="21075" windowHeight="13350" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="21075" windowHeight="13350" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
   <si>
     <t>values</t>
   </si>
@@ -57,20 +57,38 @@
     <t>pound</t>
   </si>
   <si>
-    <t>franc suisse</t>
-  </si>
-  <si>
     <t>japanese</t>
   </si>
   <si>
     <t>Korea</t>
+  </si>
+  <si>
+    <t>currency - euro</t>
+  </si>
+  <si>
+    <t>currency - NewZeland</t>
+  </si>
+  <si>
+    <t>B -Bitcoin, after</t>
+  </si>
+  <si>
+    <t>currency - Singapore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">currency -franc suisse </t>
+  </si>
+  <si>
+    <t>accounting - franc suisse</t>
+  </si>
+  <si>
+    <t>accounting- CHF allemand Liech</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="16">
+  <numFmts count="22">
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="165" formatCode="[$$-409]#,##0.00"/>
@@ -87,6 +105,12 @@
     <numFmt numFmtId="176" formatCode="#,##0.00\ [$CHF-417]"/>
     <numFmt numFmtId="177" formatCode="[$¥-411]#,##0.00"/>
     <numFmt numFmtId="178" formatCode="[$₩-412]#,##0.00"/>
+    <numFmt numFmtId="179" formatCode="#,##0\ &quot;€&quot;"/>
+    <numFmt numFmtId="180" formatCode="[$$-1409]#,##0.00"/>
+    <numFmt numFmtId="181" formatCode="#,##0.000000\ [$₿]" x16r2:formatCode16="#,##0.000000\ [$₿-x-xbt1]"/>
+    <numFmt numFmtId="182" formatCode="[$$-4809]#,##0.00"/>
+    <numFmt numFmtId="184" formatCode="_-* #,##0.00\ [$CHF-417]_-;\-* #,##0.00\ [$CHF-417]_-;_-* &quot;-&quot;??\ [$CHF-417]_-;_-@_-"/>
+    <numFmt numFmtId="185" formatCode="[$CHF-1407]\ #,##0.00;\-[$CHF-1407]\ #,##0.00"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -117,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -135,6 +159,12 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="182" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="184" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="185" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -419,10 +449,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="1" max="1" width="29" customWidth="1"/>
     <col min="2" max="2" width="24.42578125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -481,85 +511,134 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="10">
-        <v>23344</v>
+        <v>14</v>
+      </c>
+      <c r="B8" s="19">
+        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="10">
         <v>23344</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" s="11">
-        <v>12000</v>
+        <v>5</v>
+      </c>
+      <c r="B10" s="5">
+        <v>23344</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="11">
         <v>12000</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>8</v>
-      </c>
-      <c r="B12" s="8">
-        <v>456.78</v>
+        <v>6</v>
+      </c>
+      <c r="B12" s="12">
+        <v>12000</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="9">
+      <c r="B13" s="8">
         <v>456.78</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>9</v>
-      </c>
-      <c r="B14" s="13">
-        <v>344</v>
+        <v>8</v>
+      </c>
+      <c r="B14" s="9">
+        <v>456.78</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>10</v>
-      </c>
-      <c r="B15" s="14">
-        <v>345</v>
+        <v>9</v>
+      </c>
+      <c r="B15" s="13">
+        <v>344</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>11</v>
-      </c>
-      <c r="B16" s="15">
-        <v>34</v>
+        <v>16</v>
+      </c>
+      <c r="B16" s="14">
+        <v>345</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="21">
+        <v>567.89</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" s="22">
+        <v>567.89</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>10</v>
+      </c>
+      <c r="B19" s="15">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>11</v>
+      </c>
+      <c r="B20" s="16">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>12</v>
       </c>
-      <c r="B17" s="16">
-        <v>45</v>
+      <c r="B21" s="17">
+        <v>345600</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>13</v>
+      </c>
+      <c r="B22" s="18">
+        <v>9700</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>15</v>
+      </c>
+      <c r="B23" s="20">
+        <v>456</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>